<commit_message>
Update code luồng thay đổi
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/template_QTGNGL.xlsx
+++ b/Data_Product/App_Data/template_QTGNGL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA_PR\Data_Product\App_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SOFTWARE\DATA_PR\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CC7B45-443A-4418-8D7E-967FB32CF92D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B0582C-62C2-49A9-9AAF-A084A9C66BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{B537A817-926E-4385-A812-CDE5F844F19A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B537A817-926E-4385-A812-CDE5F844F19A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t xml:space="preserve">            TỔNG HỢP BẢNG DỮ LIỆU VỀ GANG LỎNG - GANG THỎI</t>
   </si>
@@ -88,6 +88,15 @@
   </si>
   <si>
     <t>Ngày luyện :……………….. - Ca :………. - Kíp :……. - Lò cao :………..</t>
+  </si>
+  <si>
+    <t>Khối lượng HRC</t>
+  </si>
+  <si>
+    <t>Khối lượng ĐÚC</t>
+  </si>
+  <si>
+    <t>Sàn ra gang</t>
   </si>
 </sst>
 </file>
@@ -147,7 +156,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -259,34 +268,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -305,6 +330,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -672,7 +703,7 @@
     <col min="3" max="3" width="23" customWidth="1"/>
     <col min="4" max="5" width="11.140625" customWidth="1"/>
     <col min="6" max="6" width="12.140625" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" customWidth="1"/>
     <col min="8" max="8" width="16.85546875" customWidth="1"/>
     <col min="9" max="9" width="18.140625" customWidth="1"/>
     <col min="10" max="10" width="20.42578125" customWidth="1"/>
@@ -681,6 +712,8 @@
     <col min="15" max="16" width="11.5703125" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" customWidth="1"/>
+    <col min="19" max="19" width="15.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -750,82 +783,94 @@
       <c r="T5" s="6"/>
     </row>
     <row r="7" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="I7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="J7" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J7" s="15" t="s">
+      <c r="K7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="L7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="L7" s="7"/>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
-      <c r="O7" s="8" t="s">
+      <c r="O7" s="7"/>
+      <c r="P7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="P7" s="9" t="s">
+      <c r="Q7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="Q7" s="9" t="s">
+      <c r="R7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="R7" s="7" t="s">
+      <c r="S7" s="11" t="s">
         <v>16</v>
+      </c>
+      <c r="T7" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="U7" s="18" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="2" t="s">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="O8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O8" s="8"/>
-      <c r="P8" s="10"/>
+      <c r="P8" s="8"/>
       <c r="Q8" s="10"/>
-      <c r="R8" s="7"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="11"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
     </row>
     <row r="9" spans="1:25" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -848,24 +893,27 @@
       <c r="R9" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="20">
+    <mergeCell ref="U7:U8"/>
     <mergeCell ref="H7:H8"/>
+    <mergeCell ref="T7:T8"/>
+    <mergeCell ref="I7:I8"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="A5:T5"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="L7:O7"/>
     <mergeCell ref="P7:P8"/>
-    <mergeCell ref="R7:R8"/>
-    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="S7:S8"/>
+    <mergeCell ref="J7:J8"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="Q7:Q8"/>
-    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="R7:R8"/>
+    <mergeCell ref="K7:K8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
+    <mergeCell ref="G7:G8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
-    <mergeCell ref="G7:G8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>